<commit_message>
Alteração de informação sobre a prioridade de cada um dos testes em caso de falha
</commit_message>
<xml_diff>
--- a/docs/Testes.xlsx
+++ b/docs/Testes.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Documents\Qa\Projeto Forge QA\qa-portifolio\projeto-01-saucedemo\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucas\Desktop\projeto-01-saucedemo\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D2093C4-2B43-4A27-B4CA-5E97D55060A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11DAF372-6625-4E95-BAD6-543BB219846F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{06FA6674-3670-4036-8892-40D7D9CB0AAF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{06FA6674-3670-4036-8892-40D7D9CB0AAF}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="97">
   <si>
     <t>ID</t>
   </si>
@@ -321,6 +321,15 @@
   </si>
   <si>
     <t>É possível fazer login e usuario vai para a home</t>
+  </si>
+  <si>
+    <t>Prioridade</t>
+  </si>
+  <si>
+    <t>Média</t>
+  </si>
+  <si>
+    <t>Alta</t>
   </si>
 </sst>
 </file>
@@ -439,10 +448,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -452,32 +479,228 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="21">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -807,45 +1030,49 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B34EEAA7-8427-4764-B765-EDB6EF24D6B8}">
-  <dimension ref="D7:N39"/>
+  <dimension ref="D7:O39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="6" max="6" width="18.88671875" customWidth="1"/>
     <col min="7" max="7" width="49" customWidth="1"/>
+    <col min="8" max="9" width="0" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="56.44140625" customWidth="1"/>
     <col min="13" max="13" width="20.77734375" customWidth="1"/>
-    <col min="14" max="14" width="16.44140625" style="12" customWidth="1"/>
+    <col min="14" max="14" width="16.44140625" style="5" customWidth="1"/>
+    <col min="15" max="15" width="9.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D7" s="7" t="s">
+    <row r="7" spans="4:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="7"/>
-      <c r="N7" s="7"/>
-    </row>
-    <row r="8" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="7"/>
-      <c r="N8" s="7"/>
-    </row>
-    <row r="9" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="12"/>
+      <c r="M7" s="12"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="12"/>
+    </row>
+    <row r="8" spans="4:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="12"/>
+      <c r="M8" s="12"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+    </row>
+    <row r="9" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D9" s="1" t="s">
         <v>0</v>
       </c>
@@ -864,758 +1091,823 @@
       </c>
       <c r="L9" s="6"/>
       <c r="M9" s="6"/>
-      <c r="N9" s="10" t="s">
+      <c r="N9" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="O9" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D10" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
-      <c r="H10" s="8" t="s">
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="3" t="s">
+      <c r="I10" s="7"/>
+      <c r="J10" s="7"/>
+      <c r="K10" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="L10" s="4"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="11" t="s">
+      <c r="L10" s="10"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="4" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="11" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="O10" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="11" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D11" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="E11" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
-      <c r="H11" s="8" t="s">
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L11" s="4"/>
-      <c r="M11" s="5"/>
-      <c r="N11" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="12" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I11" s="7"/>
+      <c r="J11" s="7"/>
+      <c r="K11" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L11" s="10"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O11" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D12" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="E12" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
-      <c r="H12" s="8" t="s">
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
+      <c r="H12" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L12" s="4"/>
-      <c r="M12" s="5"/>
-      <c r="N12" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="13" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I12" s="7"/>
+      <c r="J12" s="7"/>
+      <c r="K12" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L12" s="10"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O12" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="13" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D13" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E13" s="8" t="s">
+      <c r="E13" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8" t="s">
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="3" t="s">
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="L13" s="4"/>
-      <c r="M13" s="5"/>
-      <c r="N13" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="14" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="L13" s="10"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O13" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="14" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D14" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E14" s="8" t="s">
+      <c r="E14" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8" t="s">
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="3" t="s">
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="L14" s="4"/>
-      <c r="M14" s="5"/>
-      <c r="N14" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="15" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="L14" s="10"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O14" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D15" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="8" t="s">
+      <c r="E15" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8" t="s">
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="3" t="s">
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="L15" s="4"/>
-      <c r="M15" s="5"/>
-      <c r="N15" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="16" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="L15" s="10"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O15" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="16" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="8" t="s">
+      <c r="E16" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8" t="s">
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L16" s="4"/>
-      <c r="M16" s="5"/>
-      <c r="N16" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="17" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L16" s="10"/>
+      <c r="M16" s="11"/>
+      <c r="N16" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O16" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="17" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D17" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E17" s="8" t="s">
+      <c r="E17" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8" t="s">
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L17" s="4"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="18" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L17" s="10"/>
+      <c r="M17" s="11"/>
+      <c r="N17" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O17" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="18" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D18" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E18" s="8" t="s">
+      <c r="E18" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8" t="s">
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L18" s="4"/>
-      <c r="M18" s="5"/>
-      <c r="N18" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="19" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L18" s="10"/>
+      <c r="M18" s="11"/>
+      <c r="N18" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O18" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="19" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D19" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8" t="s">
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L19" s="4"/>
-      <c r="M19" s="5"/>
-      <c r="N19" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="20" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L19" s="10"/>
+      <c r="M19" s="11"/>
+      <c r="N19" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O19" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="20" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D20" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="8" t="s">
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L20" s="4"/>
-      <c r="M20" s="5"/>
-      <c r="N20" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="21" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I20" s="7"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L20" s="10"/>
+      <c r="M20" s="11"/>
+      <c r="N20" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O20" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D21" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="F21" s="9"/>
-      <c r="G21" s="9"/>
-      <c r="H21" s="8" t="s">
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L21" s="4"/>
-      <c r="M21" s="5"/>
-      <c r="N21" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="22" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L21" s="10"/>
+      <c r="M21" s="11"/>
+      <c r="N21" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O21" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D22" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="E22" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8" t="s">
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L22" s="4"/>
-      <c r="M22" s="5"/>
-      <c r="N22" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="23" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L22" s="10"/>
+      <c r="M22" s="11"/>
+      <c r="N22" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O22" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D23" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E23" s="8" t="s">
+      <c r="E23" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8" t="s">
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
-      <c r="K23" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L23" s="4"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="24" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L23" s="10"/>
+      <c r="M23" s="11"/>
+      <c r="N23" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O23" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D24" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E24" s="8" t="s">
+      <c r="E24" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8" t="s">
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
-      <c r="K24" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L24" s="4"/>
-      <c r="M24" s="5"/>
-      <c r="N24" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="25" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L24" s="10"/>
+      <c r="M24" s="11"/>
+      <c r="N24" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O24" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="25" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D25" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E25" s="8" t="s">
+      <c r="E25" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8" t="s">
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L25" s="4"/>
-      <c r="M25" s="5"/>
-      <c r="N25" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="26" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L25" s="10"/>
+      <c r="M25" s="11"/>
+      <c r="N25" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O25" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="26" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D26" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E26" s="8" t="s">
+      <c r="E26" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8" t="s">
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
-      <c r="K26" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L26" s="4"/>
-      <c r="M26" s="5"/>
-      <c r="N26" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="27" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L26" s="10"/>
+      <c r="M26" s="11"/>
+      <c r="N26" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O26" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="27" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D27" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E27" s="8" t="s">
+      <c r="E27" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8" t="s">
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="I27" s="8"/>
-      <c r="J27" s="8"/>
-      <c r="K27" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L27" s="4"/>
-      <c r="M27" s="5"/>
-      <c r="N27" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="28" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I27" s="7"/>
+      <c r="J27" s="7"/>
+      <c r="K27" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L27" s="10"/>
+      <c r="M27" s="11"/>
+      <c r="N27" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O27" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="28" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D28" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="E28" s="8" t="s">
+      <c r="E28" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8" t="s">
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="I28" s="8"/>
-      <c r="J28" s="8"/>
-      <c r="K28" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L28" s="4"/>
-      <c r="M28" s="5"/>
-      <c r="N28" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="29" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I28" s="7"/>
+      <c r="J28" s="7"/>
+      <c r="K28" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L28" s="10"/>
+      <c r="M28" s="11"/>
+      <c r="N28" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O28" s="13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="29" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D29" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="E29" s="8" t="s">
+      <c r="E29" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8" t="s">
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="I29" s="8"/>
-      <c r="J29" s="8"/>
-      <c r="K29" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L29" s="4"/>
-      <c r="M29" s="5"/>
-      <c r="N29" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="30" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I29" s="7"/>
+      <c r="J29" s="7"/>
+      <c r="K29" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L29" s="10"/>
+      <c r="M29" s="11"/>
+      <c r="N29" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O29" s="13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="30" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D30" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="E30" s="8" t="s">
+      <c r="E30" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
-      <c r="H30" s="8" t="s">
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="I30" s="8"/>
-      <c r="J30" s="8"/>
-      <c r="K30" s="3" t="s">
+      <c r="I30" s="7"/>
+      <c r="J30" s="7"/>
+      <c r="K30" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="L30" s="4"/>
-      <c r="M30" s="5"/>
-      <c r="N30" s="11" t="s">
+      <c r="L30" s="10"/>
+      <c r="M30" s="11"/>
+      <c r="N30" s="4" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="31" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="O30" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="31" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D31" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E31" s="8" t="s">
+      <c r="E31" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
-      <c r="H31" s="8" t="s">
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="I31" s="8"/>
-      <c r="J31" s="8"/>
-      <c r="K31" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L31" s="4"/>
-      <c r="M31" s="5"/>
-      <c r="N31" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="32" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+      <c r="K31" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L31" s="10"/>
+      <c r="M31" s="11"/>
+      <c r="N31" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O31" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D32" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="E32" s="8" t="s">
+      <c r="E32" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
-      <c r="H32" s="8" t="s">
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
+      <c r="H32" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="I32" s="8"/>
-      <c r="J32" s="8"/>
-      <c r="K32" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L32" s="4"/>
-      <c r="M32" s="5"/>
-      <c r="N32" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="33" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I32" s="7"/>
+      <c r="J32" s="7"/>
+      <c r="K32" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L32" s="10"/>
+      <c r="M32" s="11"/>
+      <c r="N32" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O32" s="13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="33" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D33" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E33" s="8" t="s">
+      <c r="E33" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
-      <c r="H33" s="8" t="s">
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="I33" s="8"/>
-      <c r="J33" s="8"/>
-      <c r="K33" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L33" s="4"/>
-      <c r="M33" s="5"/>
-      <c r="N33" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="34" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I33" s="7"/>
+      <c r="J33" s="7"/>
+      <c r="K33" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L33" s="10"/>
+      <c r="M33" s="11"/>
+      <c r="N33" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O33" s="13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="34" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D34" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="E34" s="8" t="s">
+      <c r="E34" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
-      <c r="H34" s="8" t="s">
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
+      <c r="H34" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="I34" s="8"/>
-      <c r="J34" s="8"/>
-      <c r="K34" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L34" s="4"/>
-      <c r="M34" s="5"/>
-      <c r="N34" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="35" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I34" s="7"/>
+      <c r="J34" s="7"/>
+      <c r="K34" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L34" s="10"/>
+      <c r="M34" s="11"/>
+      <c r="N34" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O34" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="35" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D35" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="E35" s="8" t="s">
+      <c r="E35" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
-      <c r="H35" s="8" t="s">
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
+      <c r="H35" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="I35" s="8"/>
-      <c r="J35" s="8"/>
-      <c r="K35" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L35" s="4"/>
-      <c r="M35" s="5"/>
-      <c r="N35" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="36" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I35" s="7"/>
+      <c r="J35" s="7"/>
+      <c r="K35" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L35" s="10"/>
+      <c r="M35" s="11"/>
+      <c r="N35" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O35" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D36" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E36" s="8" t="s">
+      <c r="E36" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
-      <c r="H36" s="8" t="s">
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+      <c r="H36" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="I36" s="8"/>
-      <c r="J36" s="8"/>
-      <c r="K36" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="L36" s="4"/>
-      <c r="M36" s="5"/>
-      <c r="N36" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="37" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="I36" s="7"/>
+      <c r="J36" s="7"/>
+      <c r="K36" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="L36" s="10"/>
+      <c r="M36" s="11"/>
+      <c r="N36" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="O36" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="37" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D37" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="E37" s="8" t="s">
+      <c r="E37" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
-      <c r="H37" s="8" t="s">
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+      <c r="H37" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I37" s="8"/>
-      <c r="J37" s="8"/>
-      <c r="K37" s="3" t="s">
+      <c r="I37" s="7"/>
+      <c r="J37" s="7"/>
+      <c r="K37" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="L37" s="4"/>
-      <c r="M37" s="5"/>
-      <c r="N37" s="11" t="s">
+      <c r="L37" s="10"/>
+      <c r="M37" s="11"/>
+      <c r="N37" s="4" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="38" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="O37" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D38" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="E38" s="8" t="s">
+      <c r="E38" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
-      <c r="H38" s="8" t="s">
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+      <c r="H38" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="I38" s="8"/>
-      <c r="J38" s="8"/>
-      <c r="K38" s="3" t="s">
+      <c r="I38" s="7"/>
+      <c r="J38" s="7"/>
+      <c r="K38" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="L38" s="4"/>
-      <c r="M38" s="5"/>
-      <c r="N38" s="11" t="s">
+      <c r="L38" s="10"/>
+      <c r="M38" s="11"/>
+      <c r="N38" s="4" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="39" spans="4:14" x14ac:dyDescent="0.3">
+      <c r="O38" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="39" spans="4:15" x14ac:dyDescent="0.3">
       <c r="D39" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="E39" s="8" t="s">
+      <c r="E39" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
-      <c r="H39" s="8" t="s">
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+      <c r="H39" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="I39" s="8"/>
-      <c r="J39" s="8"/>
-      <c r="K39" s="3" t="s">
+      <c r="I39" s="7"/>
+      <c r="J39" s="7"/>
+      <c r="K39" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="L39" s="4"/>
-      <c r="M39" s="5"/>
-      <c r="N39" s="11" t="s">
+      <c r="L39" s="10"/>
+      <c r="M39" s="11"/>
+      <c r="N39" s="4" t="s">
         <v>83</v>
+      </c>
+      <c r="O39" s="13" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="94">
-    <mergeCell ref="E9:G9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="E12:G12"/>
-    <mergeCell ref="H12:J12"/>
-    <mergeCell ref="E20:G20"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="E21:G21"/>
-    <mergeCell ref="H21:J21"/>
-    <mergeCell ref="E16:G16"/>
-    <mergeCell ref="H16:J16"/>
-    <mergeCell ref="E17:G17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="E22:G22"/>
-    <mergeCell ref="H22:J22"/>
-    <mergeCell ref="E23:G23"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="E24:G24"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="E25:G25"/>
-    <mergeCell ref="H25:J25"/>
-    <mergeCell ref="E26:G26"/>
-    <mergeCell ref="H26:J26"/>
-    <mergeCell ref="E27:G27"/>
-    <mergeCell ref="H27:J27"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="H28:J28"/>
-    <mergeCell ref="E29:G29"/>
-    <mergeCell ref="H29:J29"/>
-    <mergeCell ref="E30:G30"/>
-    <mergeCell ref="H30:J30"/>
-    <mergeCell ref="E31:G31"/>
-    <mergeCell ref="H31:J31"/>
-    <mergeCell ref="E32:G32"/>
-    <mergeCell ref="H32:J32"/>
-    <mergeCell ref="E33:G33"/>
-    <mergeCell ref="H33:J33"/>
-    <mergeCell ref="E34:G34"/>
-    <mergeCell ref="H34:J34"/>
-    <mergeCell ref="E35:G35"/>
-    <mergeCell ref="H35:J35"/>
-    <mergeCell ref="E36:G36"/>
-    <mergeCell ref="H36:J36"/>
-    <mergeCell ref="E37:G37"/>
-    <mergeCell ref="H37:J37"/>
-    <mergeCell ref="E38:G38"/>
-    <mergeCell ref="H38:J38"/>
-    <mergeCell ref="E39:G39"/>
-    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="D7:O8"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="K39:M39"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="K31:M31"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="K21:M21"/>
+    <mergeCell ref="K22:M22"/>
+    <mergeCell ref="K23:M23"/>
+    <mergeCell ref="K24:M24"/>
+    <mergeCell ref="K25:M25"/>
+    <mergeCell ref="K26:M26"/>
+    <mergeCell ref="K27:M27"/>
+    <mergeCell ref="K28:M28"/>
+    <mergeCell ref="K29:M29"/>
+    <mergeCell ref="K30:M30"/>
+    <mergeCell ref="K14:M14"/>
+    <mergeCell ref="K15:M15"/>
+    <mergeCell ref="K16:M16"/>
+    <mergeCell ref="K17:M17"/>
+    <mergeCell ref="K18:M18"/>
     <mergeCell ref="K19:M19"/>
     <mergeCell ref="K9:M9"/>
-    <mergeCell ref="D7:N8"/>
     <mergeCell ref="K10:M10"/>
     <mergeCell ref="K11:M11"/>
     <mergeCell ref="K12:M12"/>
@@ -1629,38 +1921,130 @@
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="H15:J15"/>
     <mergeCell ref="E10:G10"/>
-    <mergeCell ref="K14:M14"/>
-    <mergeCell ref="K15:M15"/>
-    <mergeCell ref="K16:M16"/>
-    <mergeCell ref="K17:M17"/>
-    <mergeCell ref="K18:M18"/>
-    <mergeCell ref="K31:M31"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="K21:M21"/>
-    <mergeCell ref="K22:M22"/>
-    <mergeCell ref="K23:M23"/>
-    <mergeCell ref="K24:M24"/>
-    <mergeCell ref="K25:M25"/>
-    <mergeCell ref="K26:M26"/>
-    <mergeCell ref="K27:M27"/>
-    <mergeCell ref="K28:M28"/>
-    <mergeCell ref="K29:M29"/>
-    <mergeCell ref="K30:M30"/>
-    <mergeCell ref="K38:M38"/>
-    <mergeCell ref="K39:M39"/>
-    <mergeCell ref="K32:M32"/>
-    <mergeCell ref="K33:M33"/>
-    <mergeCell ref="K34:M34"/>
-    <mergeCell ref="K35:M35"/>
-    <mergeCell ref="K36:M36"/>
-    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="H37:J37"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="E39:G39"/>
+    <mergeCell ref="H39:J39"/>
+    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="H34:J34"/>
+    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="H35:J35"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="E31:G31"/>
+    <mergeCell ref="H31:J31"/>
+    <mergeCell ref="E32:G32"/>
+    <mergeCell ref="H32:J32"/>
+    <mergeCell ref="E33:G33"/>
+    <mergeCell ref="H33:J33"/>
+    <mergeCell ref="E28:G28"/>
+    <mergeCell ref="H28:J28"/>
+    <mergeCell ref="E29:G29"/>
+    <mergeCell ref="H29:J29"/>
+    <mergeCell ref="E30:G30"/>
+    <mergeCell ref="H30:J30"/>
+    <mergeCell ref="E25:G25"/>
+    <mergeCell ref="H25:J25"/>
+    <mergeCell ref="E26:G26"/>
+    <mergeCell ref="H26:J26"/>
+    <mergeCell ref="E27:G27"/>
+    <mergeCell ref="H27:J27"/>
+    <mergeCell ref="E22:G22"/>
+    <mergeCell ref="H22:J22"/>
+    <mergeCell ref="E23:G23"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="E24:G24"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="E20:G20"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="E21:G21"/>
+    <mergeCell ref="H21:J21"/>
+    <mergeCell ref="E16:G16"/>
+    <mergeCell ref="H16:J16"/>
+    <mergeCell ref="E17:G17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="E18:G18"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="H11:J11"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations count="1">
+  <conditionalFormatting sqref="O10:O39">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="formula" val="&quot;Alta&quot;"/>
+        <cfvo type="formula" val="&quot;Media&quot;"/>
+        <cfvo type="formula" val="&quot;Baixa&quot;"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="dataBar" priority="7">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF555A"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{B1D3A6B3-12FD-42E4-ADD2-D66CAC69ED57}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="6" operator="containsText" text="Baixa">
+      <formula>NOT(ISERROR(SEARCH("Baixa",O10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="Média">
+      <formula>NOT(ISERROR(SEARCH("Média",O10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="8" priority="4" operator="containsText" text="Alta">
+      <formula>NOT(ISERROR(SEARCH("Alta",O10)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N10:N39">
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="Aprovado">
+      <formula>NOT(ISERROR(SEARCH("Aprovado",N10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="Reprovado">
+      <formula>NOT(ISERROR(SEARCH("Reprovado",N10)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Bloqueado">
+      <formula>NOT(ISERROR(SEARCH("Bloqueado",N10)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="N9:N39" xr:uid="{0CEAD779-7FEC-41AD-9780-350030E61AC9}">
       <formula1>"Aprovado, Reprovado, Bloqueado, Não executado"</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O10:O39" xr:uid="{8A769397-3517-4CDB-8E4A-CCD22FE02B4C}">
+      <formula1>"Baixa, Média, Alta,"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{B1D3A6B3-12FD-42E4-ADD2-D66CAC69ED57}">
+            <x14:dataBar minLength="0" maxLength="100" gradient="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>O10:O39</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>